<commit_message>
Implement specialized login verification, overhaul sportsbook registration adapters, and clean false positive records
</commit_message>
<xml_diff>
--- a/Test.xlsx
+++ b/Test.xlsx
@@ -52692,7 +52692,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
@@ -52722,413 +52722,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="0" t="inlineStr">
-        <is>
-          <t>Courtney Weaver</t>
-        </is>
-      </c>
-      <c r="B2" s="0" t="inlineStr">
-        <is>
-          <t>Fairplay Bet</t>
-        </is>
-      </c>
-      <c r="C2" s="0" t="inlineStr">
-        <is>
-          <t>courtney.weaver.5580@gmail.com</t>
-        </is>
-      </c>
-      <c r="D2" s="0" t="inlineStr">
-        <is>
-          <t>courtney.weaver.5580@gmail.com</t>
-        </is>
-      </c>
-      <c r="E2" s="0" t="inlineStr">
-        <is>
-          <t>LXElC#9W62WlfK</t>
-        </is>
-      </c>
-      <c r="F2" s="0" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:35:32</t>
-        </is>
-      </c>
-      <c r="G2" s="0" t="inlineStr">
-        <is>
-          <t>FairplayBet-Direct</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="0" t="inlineStr">
-        <is>
-          <t>Daniel Buckley</t>
-        </is>
-      </c>
-      <c r="B3" s="0" t="inlineStr">
-        <is>
-          <t>Fairplay Bet</t>
-        </is>
-      </c>
-      <c r="C3" s="0" t="inlineStr">
-        <is>
-          <t>daniel.buckley.6491@gmail.com</t>
-        </is>
-      </c>
-      <c r="D3" s="0" t="inlineStr">
-        <is>
-          <t>daniel.buckley.6491@gmail.com</t>
-        </is>
-      </c>
-      <c r="E3" s="0" t="inlineStr">
-        <is>
-          <t>ataj8$fS*U%Yb5</t>
-        </is>
-      </c>
-      <c r="F3" s="0" t="inlineStr">
-        <is>
-          <t>2026-08-21 07:38:00</t>
-        </is>
-      </c>
-      <c r="G3" s="0" t="inlineStr">
-        <is>
-          <t>FairplayBet-Direct</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="0" t="inlineStr">
-        <is>
-          <t>Leoni kay Samuda</t>
-        </is>
-      </c>
-      <c r="B4" s="0" t="inlineStr">
-        <is>
-          <t>Fairplay Bet</t>
-        </is>
-      </c>
-      <c r="C4" s="0" t="inlineStr">
-        <is>
-          <t>leoni.kaysamuda.2911@gmail.com</t>
-        </is>
-      </c>
-      <c r="D4" s="0" t="inlineStr">
-        <is>
-          <t>leoni.kaysamuda.2911@gmail.com</t>
-        </is>
-      </c>
-      <c r="E4" s="0" t="inlineStr">
-        <is>
-          <t>Rq^Brvx2rgiU9N</t>
-        </is>
-      </c>
-      <c r="F4" s="0" t="inlineStr">
-        <is>
-          <t>2026-08-21 08:13:04</t>
-        </is>
-      </c>
-      <c r="G4" s="0" t="inlineStr">
-        <is>
-          <t>FairplayBet-Direct</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="0" t="inlineStr">
-        <is>
-          <t>Laura Allen</t>
-        </is>
-      </c>
-      <c r="B5" s="0" t="inlineStr">
-        <is>
-          <t>Fairplay Bet</t>
-        </is>
-      </c>
-      <c r="C5" s="0" t="inlineStr">
-        <is>
-          <t>lauallen76@gmail.com</t>
-        </is>
-      </c>
-      <c r="D5" s="0" t="inlineStr">
-        <is>
-          <t>lauallen76@gmail.com</t>
-        </is>
-      </c>
-      <c r="E5" s="0" t="inlineStr">
-        <is>
-          <t>MOiZCT%3DJT5uw</t>
-        </is>
-      </c>
-      <c r="F5" s="0" t="inlineStr">
-        <is>
-          <t>2026-08-21 08:45:34</t>
-        </is>
-      </c>
-      <c r="G5" s="0" t="inlineStr">
-        <is>
-          <t>FairplayBet-Direct</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="0" t="inlineStr">
-        <is>
-          <t>Kiran Bokil</t>
-        </is>
-      </c>
-      <c r="B6" s="0" t="inlineStr">
-        <is>
-          <t>Fairplay Bet</t>
-        </is>
-      </c>
-      <c r="C6" s="0" t="inlineStr">
-        <is>
-          <t>kiran.bokil88@gmail.com</t>
-        </is>
-      </c>
-      <c r="D6" s="0" t="inlineStr">
-        <is>
-          <t>kiran.bokil88@gmail.com</t>
-        </is>
-      </c>
-      <c r="E6" s="0" t="inlineStr">
-        <is>
-          <t>JIpR8C@GbbUZFs</t>
-        </is>
-      </c>
-      <c r="F6" s="0" t="inlineStr">
-        <is>
-          <t>2026-08-21 08:45:50</t>
-        </is>
-      </c>
-      <c r="G6" s="0" t="inlineStr">
-        <is>
-          <t>FairplayBet-Direct</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="0" t="inlineStr">
-        <is>
-          <t>Laura Allen</t>
-        </is>
-      </c>
-      <c r="B7" s="0" t="inlineStr">
-        <is>
-          <t>Betgoodwin</t>
-        </is>
-      </c>
-      <c r="C7" s="0" t="inlineStr">
-        <is>
-          <t>lauallen76@gmail.com</t>
-        </is>
-      </c>
-      <c r="D7" s="0" t="inlineStr">
-        <is>
-          <t>lauallen76@gmail.com</t>
-        </is>
-      </c>
-      <c r="E7" s="0" t="inlineStr">
-        <is>
-          <t>AeE&amp;T3q!#GL$#9</t>
-        </is>
-      </c>
-      <c r="F7" s="0" t="inlineStr">
-        <is>
-          <t>2026-08-21 13:04:27</t>
-        </is>
-      </c>
-      <c r="G7" s="0" t="inlineStr">
-        <is>
-          <t>Betgoodwin-Direct</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="0" t="inlineStr">
-        <is>
-          <t>Kiran Bokil</t>
-        </is>
-      </c>
-      <c r="B8" s="0" t="inlineStr">
-        <is>
-          <t>Betting Lounge #1 (Bet St George)</t>
-        </is>
-      </c>
-      <c r="C8" s="0" t="inlineStr">
-        <is>
-          <t>kiran.bokil88@gmail.com</t>
-        </is>
-      </c>
-      <c r="D8" s="0" t="inlineStr">
-        <is>
-          <t>kiran.bokil88@gmail.com</t>
-        </is>
-      </c>
-      <c r="E8" s="0" t="inlineStr">
-        <is>
-          <t>ED@s3pfZbNdMlc</t>
-        </is>
-      </c>
-      <c r="F8" s="0" t="inlineStr">
-        <is>
-          <t>2026-08-21 13:06:43</t>
-        </is>
-      </c>
-      <c r="G8" s="0" t="inlineStr">
-        <is>
-          <t>Betting Lounge #1 (Bet St George)-Direct</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="0" t="inlineStr">
-        <is>
-          <t>Laura Francis</t>
-        </is>
-      </c>
-      <c r="B9" s="0" t="inlineStr">
-        <is>
-          <t>Planet Sport Bet</t>
-        </is>
-      </c>
-      <c r="C9" s="0" t="inlineStr">
-        <is>
-          <t>lau.francis23@outlook.com</t>
-        </is>
-      </c>
-      <c r="D9" s="0" t="inlineStr">
-        <is>
-          <t>lau.francis23@outlook.com</t>
-        </is>
-      </c>
-      <c r="E9" s="0" t="inlineStr">
-        <is>
-          <t>t5BV6*I8eugNS8</t>
-        </is>
-      </c>
-      <c r="F9" s="0" t="inlineStr">
-        <is>
-          <t>2026-08-21 13:09:42</t>
-        </is>
-      </c>
-      <c r="G9" s="0" t="inlineStr">
-        <is>
-          <t>PlanetSportBet-Direct</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="0" t="inlineStr">
-        <is>
-          <t>Gabriella Dutton</t>
-        </is>
-      </c>
-      <c r="B10" s="0" t="inlineStr">
-        <is>
-          <t>BresBet</t>
-        </is>
-      </c>
-      <c r="C10" s="0" t="inlineStr">
-        <is>
-          <t>ella.dutton95@outlook.com</t>
-        </is>
-      </c>
-      <c r="D10" s="0" t="inlineStr">
-        <is>
-          <t>ella.dutton95@outlook.com</t>
-        </is>
-      </c>
-      <c r="E10" s="0" t="inlineStr">
-        <is>
-          <t>L#9mIRp2hCyH$3</t>
-        </is>
-      </c>
-      <c r="F10" s="0" t="inlineStr">
-        <is>
-          <t>2026-08-21 13:10:06</t>
-        </is>
-      </c>
-      <c r="G10" s="0" t="inlineStr">
-        <is>
-          <t>BresBet-Direct</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="0" t="inlineStr">
-        <is>
-          <t>Bobbie Shortland</t>
-        </is>
-      </c>
-      <c r="B11" s="0" t="inlineStr">
-        <is>
-          <t>Star Sports</t>
-        </is>
-      </c>
-      <c r="C11" s="0" t="inlineStr">
-        <is>
-          <t>bobb.shortland19@gmail.com</t>
-        </is>
-      </c>
-      <c r="D11" s="0" t="inlineStr">
-        <is>
-          <t>bobb.shortland19@gmail.com</t>
-        </is>
-      </c>
-      <c r="E11" s="0" t="inlineStr">
-        <is>
-          <t>jk#J9d1yyONmJ1</t>
-        </is>
-      </c>
-      <c r="F11" s="0" t="inlineStr">
-        <is>
-          <t>2026-08-21 13:11:48</t>
-        </is>
-      </c>
-      <c r="G11" s="0" t="inlineStr">
-        <is>
-          <t>StarSports-Direct</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Shannon Grover</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>QuinnBet</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>shannon.grover27@outlook.com</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>shannon.grover27@outlook.com</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Q7UB4oaD9D^X!O</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>2026-08-21 13:12:06</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>QuinnBet-Direct</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: enhance duplicate detection across bookmakers, add Betgoodwin & PlanetSportBet adapters, sanitize address data, and streamline failure recovery
</commit_message>
<xml_diff>
--- a/Test.xlsx
+++ b/Test.xlsx
@@ -52692,7 +52692,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
@@ -52722,6 +52722,1038 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>Jake Fox</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>Fairplay Bet</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>jake.fox93@gmail.com</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>jake.fox93@gmail.com</t>
+        </is>
+      </c>
+      <c r="E2" s="0" t="inlineStr">
+        <is>
+          <t>Ro#etLXG9cy8Px</t>
+        </is>
+      </c>
+      <c r="F2" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-22 21:48:32</t>
+        </is>
+      </c>
+      <c r="G2" s="0" t="inlineStr">
+        <is>
+          <t>FairplayBet-Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>Hannah Parkin</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>Fairplay Bet</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>hannahhoney8@gmail.com</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>hannahhoney8@gmail.com</t>
+        </is>
+      </c>
+      <c r="E3" s="0" t="inlineStr">
+        <is>
+          <t>jSoh#8$wDeHoOz</t>
+        </is>
+      </c>
+      <c r="F3" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-22 21:49:01</t>
+        </is>
+      </c>
+      <c r="G3" s="0" t="inlineStr">
+        <is>
+          <t>FairplayBet-Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>Courtney Weaver</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>Betfred</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>courtney.weaver.5580@gmail.com</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>courtney.weaver.5580@gmail.com</t>
+        </is>
+      </c>
+      <c r="E4" s="0" t="inlineStr">
+        <is>
+          <t>D6s*0yk9cyAVp5</t>
+        </is>
+      </c>
+      <c r="F4" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-22 22:07:25</t>
+        </is>
+      </c>
+      <c r="G4" s="0" t="inlineStr">
+        <is>
+          <t>Betfred-Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>Daniel Buckley</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>Betfred</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>daniel.buckley.6491@gmail.com</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>daniel.buckley.6491@gmail.com</t>
+        </is>
+      </c>
+      <c r="E5" s="0" t="inlineStr">
+        <is>
+          <t>F4xF@7dgUIF8$w</t>
+        </is>
+      </c>
+      <c r="F5" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-22 22:08:07</t>
+        </is>
+      </c>
+      <c r="G5" s="0" t="inlineStr">
+        <is>
+          <t>Betfred-Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>Leoni kay Samuda</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>Betfred</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>leoni.kaysamuda.2911@gmail.com</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>leoni.kaysamuda.2911@gmail.com</t>
+        </is>
+      </c>
+      <c r="E6" s="0" t="inlineStr">
+        <is>
+          <t>m0q9#p$dmOG!T*</t>
+        </is>
+      </c>
+      <c r="F6" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-22 22:08:47</t>
+        </is>
+      </c>
+      <c r="G6" s="0" t="inlineStr">
+        <is>
+          <t>Betfred-Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>Laura Francis</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>Betfred</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>lau.francis23@outlook.com</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>lau.francis23@outlook.com</t>
+        </is>
+      </c>
+      <c r="E7" s="0" t="inlineStr">
+        <is>
+          <t>OJ#SvF6kFbb$8I</t>
+        </is>
+      </c>
+      <c r="F7" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-22 22:09:46</t>
+        </is>
+      </c>
+      <c r="G7" s="0" t="inlineStr">
+        <is>
+          <t>Betfred-Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>Laura Allen</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>Betfred</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>lauallen76@gmail.com</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>lauallen76@gmail.com</t>
+        </is>
+      </c>
+      <c r="E8" s="0" t="inlineStr">
+        <is>
+          <t>ocDaZvh$%9$CoU</t>
+        </is>
+      </c>
+      <c r="F8" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-22 22:25:54</t>
+        </is>
+      </c>
+      <c r="G8" s="0" t="inlineStr">
+        <is>
+          <t>Betfred-Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>Gabriella Dutton</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>Betfred</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>ella.dutton95@outlook.com</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>ella.dutton95@outlook.com</t>
+        </is>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t>p5S1t5L5@3e4E$</t>
+        </is>
+      </c>
+      <c r="F9" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-22 22:43:48</t>
+        </is>
+      </c>
+      <c r="G9" s="0" t="inlineStr">
+        <is>
+          <t>Betfred-Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>Bobbie Shortland</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>Betfred</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>bobb.shortland19@gmail.com</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>bobb.shortland19@gmail.com</t>
+        </is>
+      </c>
+      <c r="E10" s="0" t="inlineStr">
+        <is>
+          <t>fLS$%I7e%d8b$J</t>
+        </is>
+      </c>
+      <c r="F10" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-22 22:44:32</t>
+        </is>
+      </c>
+      <c r="G10" s="0" t="inlineStr">
+        <is>
+          <t>Betfred-Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>Shannon Grover</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>Betfred</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>shannon.grover27@outlook.com</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>shannon.grover27@outlook.com</t>
+        </is>
+      </c>
+      <c r="E11" s="0" t="inlineStr">
+        <is>
+          <t>4ZkO8#wkFTjxt0</t>
+        </is>
+      </c>
+      <c r="F11" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-22 22:50:31</t>
+        </is>
+      </c>
+      <c r="G11" s="0" t="inlineStr">
+        <is>
+          <t>Betfred-Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>Jake Fox</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>Betfred</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>jake.fox93@gmail.com</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>jake.fox93@gmail.com</t>
+        </is>
+      </c>
+      <c r="E12" s="0" t="inlineStr">
+        <is>
+          <t>5*hHe4B1c^Vtn5</t>
+        </is>
+      </c>
+      <c r="F12" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-22 22:50:49</t>
+        </is>
+      </c>
+      <c r="G12" s="0" t="inlineStr">
+        <is>
+          <t>Betfred-Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>Hannah Parkin</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>Betfred</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>hannahhoney8@gmail.com</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>hannahhoney8@gmail.com</t>
+        </is>
+      </c>
+      <c r="E13" s="0" t="inlineStr">
+        <is>
+          <t>t%3V3y6paYlkW!</t>
+        </is>
+      </c>
+      <c r="F13" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-22 22:51:11</t>
+        </is>
+      </c>
+      <c r="G13" s="0" t="inlineStr">
+        <is>
+          <t>Betfred-Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>Helen Cassels</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>Betfred</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>helen.cassels05@outlook.com</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>helen.cassels05@outlook.com</t>
+        </is>
+      </c>
+      <c r="E14" s="0" t="inlineStr">
+        <is>
+          <t>mzhoIGW2$qP8ui</t>
+        </is>
+      </c>
+      <c r="F14" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-22 22:51:51</t>
+        </is>
+      </c>
+      <c r="G14" s="0" t="inlineStr">
+        <is>
+          <t>Betfred-Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>Debbie Dolby</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>Betfred</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>debbie.dolby87@gmail.com</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>debbie.dolby87@gmail.com</t>
+        </is>
+      </c>
+      <c r="E15" s="0" t="inlineStr">
+        <is>
+          <t>Of4P*zLYXb&amp;5^f</t>
+        </is>
+      </c>
+      <c r="F15" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-22 22:52:36</t>
+        </is>
+      </c>
+      <c r="G15" s="0" t="inlineStr">
+        <is>
+          <t>Betfred-Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>Pritthijit Datta</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>Betfred</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>pritt.datta75@outlook.com</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>pritt.datta75@outlook.com</t>
+        </is>
+      </c>
+      <c r="E16" s="0" t="inlineStr">
+        <is>
+          <t>09L9Xkl9&amp;8uTaR</t>
+        </is>
+      </c>
+      <c r="F16" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-22 22:54:53</t>
+        </is>
+      </c>
+      <c r="G16" s="0" t="inlineStr">
+        <is>
+          <t>Betfred-Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>Kiran Bokil</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>Betfred</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>kiran.bokil88@gmail.com</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>kiran.bokil88@gmail.com</t>
+        </is>
+      </c>
+      <c r="E17" s="0" t="inlineStr">
+        <is>
+          <t>ysk48!sM6Yp$4d</t>
+        </is>
+      </c>
+      <c r="F17" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-22 22:55:32</t>
+        </is>
+      </c>
+      <c r="G17" s="0" t="inlineStr">
+        <is>
+          <t>Betfred-Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>Leoni kay Samuda</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>BresBet</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>leoni.kaysamuda.2911@gmail.com</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>leoni.kaysamuda.2911@gmail.com</t>
+        </is>
+      </c>
+      <c r="E18" s="0" t="inlineStr">
+        <is>
+          <t>rjz$#joUkXi3&amp;z</t>
+        </is>
+      </c>
+      <c r="F18" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-22 22:57:58</t>
+        </is>
+      </c>
+      <c r="G18" s="0" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>Gabriella Dutton</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>Betgoodwin</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>ella.dutton95@outlook.com</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>ella.dutton95@outlook.com</t>
+        </is>
+      </c>
+      <c r="E19" s="0" t="inlineStr">
+        <is>
+          <t>niq7Z4OcZl0Rq#</t>
+        </is>
+      </c>
+      <c r="F19" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-22 23:50:32</t>
+        </is>
+      </c>
+      <c r="G19" s="0" t="inlineStr">
+        <is>
+          <t>Betgoodwin-Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>Shannon Grover</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>Betgoodwin</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>shannon.grover27@outlook.com</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>shannon.grover27@outlook.com</t>
+        </is>
+      </c>
+      <c r="E20" s="0" t="inlineStr">
+        <is>
+          <t>PLc*k8y0H^DjyL</t>
+        </is>
+      </c>
+      <c r="F20" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-22 23:52:37</t>
+        </is>
+      </c>
+      <c r="G20" s="0" t="inlineStr">
+        <is>
+          <t>Betgoodwin-Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>Jake Fox</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>Betgoodwin</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>jake.fox93@gmail.com</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>jake.fox93@gmail.com</t>
+        </is>
+      </c>
+      <c r="E21" s="0" t="inlineStr">
+        <is>
+          <t>Ok5!&amp;5W1kH@0C4</t>
+        </is>
+      </c>
+      <c r="F21" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-22 23:53:31</t>
+        </is>
+      </c>
+      <c r="G21" s="0" t="inlineStr">
+        <is>
+          <t>Betgoodwin-Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>Hannah Parkin</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>Betgoodwin</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>hannahhoney8@gmail.com</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>hannahhoney8@gmail.com</t>
+        </is>
+      </c>
+      <c r="E22" s="0" t="inlineStr">
+        <is>
+          <t>eVH8xN1QLk#mV7</t>
+        </is>
+      </c>
+      <c r="F22" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-23 00:00:57</t>
+        </is>
+      </c>
+      <c r="G22" s="0" t="inlineStr">
+        <is>
+          <t>Betgoodwin-Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>Helen Cassels</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>Betgoodwin</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>helen.cassels05@outlook.com</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>helen.cassels05@outlook.com</t>
+        </is>
+      </c>
+      <c r="E23" s="0" t="inlineStr">
+        <is>
+          <t>3qT$t^%@5XPe89</t>
+        </is>
+      </c>
+      <c r="F23" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-23 00:01:51</t>
+        </is>
+      </c>
+      <c r="G23" s="0" t="inlineStr">
+        <is>
+          <t>Betgoodwin-Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>Debbie Dolby</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>Betgoodwin</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>debbie.dolby87@gmail.com</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>debbie.dolby87@gmail.com</t>
+        </is>
+      </c>
+      <c r="E24" s="0" t="inlineStr">
+        <is>
+          <t>bkcRGu$9Y8xkRH</t>
+        </is>
+      </c>
+      <c r="F24" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-23 00:02:45</t>
+        </is>
+      </c>
+      <c r="G24" s="0" t="inlineStr">
+        <is>
+          <t>Betgoodwin-Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>Pritthijit Datta</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>Betgoodwin</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>pritt.datta75@outlook.com</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>pritt.datta75@outlook.com</t>
+        </is>
+      </c>
+      <c r="E25" s="0" t="inlineStr">
+        <is>
+          <t>kEL#nCy6F5iCF$</t>
+        </is>
+      </c>
+      <c r="F25" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-23 00:11:38</t>
+        </is>
+      </c>
+      <c r="G25" s="0" t="inlineStr">
+        <is>
+          <t>Betgoodwin-Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>Laura Francis</t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>Betgoodwin</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>lau.francis23@outlook.com</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>lau.francis23@outlook.com</t>
+        </is>
+      </c>
+      <c r="E26" s="0" t="inlineStr">
+        <is>
+          <t>@EKW2Ivs4K7w$c</t>
+        </is>
+      </c>
+      <c r="F26" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-23 00:23:15</t>
+        </is>
+      </c>
+      <c r="G26" s="0" t="inlineStr">
+        <is>
+          <t>Betgoodwin-Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>Laura Allen</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>Betgoodwin</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>lauallen76@gmail.com</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>lauallen76@gmail.com</t>
+        </is>
+      </c>
+      <c r="E27" s="0" t="inlineStr">
+        <is>
+          <t>DnbQuC034yb*tn</t>
+        </is>
+      </c>
+      <c r="F27" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-23 00:25:23</t>
+        </is>
+      </c>
+      <c r="G27" s="0" t="inlineStr">
+        <is>
+          <t>Betgoodwin-Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>Daniel Buckley</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>Planet Sport Bet</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>daniel.buckley.6491@gmail.com</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>daniel.buckley.6491@gmail.com</t>
+        </is>
+      </c>
+      <c r="E28" s="0" t="inlineStr">
+        <is>
+          <t>xlfFId43&amp;VHYSD</t>
+        </is>
+      </c>
+      <c r="F28" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-23 00:59:06</t>
+        </is>
+      </c>
+      <c r="G28" s="0" t="inlineStr">
+        <is>
+          <t>PlanetSportBet-Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Courtney Weaver</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Planet Sport Bet</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>courtney.weaver.5580@gmail.com</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>courtney.weaver.5580@gmail.com</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>$7!7$ftO20JTtQ</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2026-08-23 00:59:57</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>PlanetSportBet-Existing</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>